<commit_message>
Add model-specific chat template handling, update results
</commit_message>
<xml_diff>
--- a/debug/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Llama-3.1-8B-Instruct/aae/total_votes_file.xlsx
+++ b/debug/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Llama-3.1-8B-Instruct/aae/total_votes_file.xlsx
@@ -430,16 +430,16 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D2">
-        <v>8</v>
+        <v>155</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="G2">
-        <v>404</v>
+        <v>204</v>
       </c>
       <c r="H2">
         <v>426</v>
@@ -450,16 +450,16 @@
         <v>8</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D3">
-        <v>11</v>
+        <v>161</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="G3">
-        <v>404</v>
+        <v>183</v>
       </c>
       <c r="H3">
         <v>426</v>

</xml_diff>

<commit_message>
Add results from rerun with new answser extraction function
</commit_message>
<xml_diff>
--- a/debug/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Llama-3.1-8B-Instruct/aae/total_votes_file.xlsx
+++ b/debug/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Llama-3.1-8B-Instruct/aae/total_votes_file.xlsx
@@ -430,16 +430,16 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D2">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="E2">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="G2">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="H2">
         <v>426</v>
@@ -450,16 +450,16 @@
         <v>8</v>
       </c>
       <c r="C3">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="D3">
-        <v>161</v>
+        <v>136</v>
       </c>
       <c r="E3">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G3">
-        <v>183</v>
+        <v>217</v>
       </c>
       <c r="H3">
         <v>426</v>

</xml_diff>